<commit_message>
Finalize Monroe/Keys inputs (tax, insurance) and add Keys section to report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xw5JeBLbuwioE3FbfVFAqz
</commit_message>
<xml_diff>
--- a/str-deal-search/STR_DSCR_Analysis.xlsx
+++ b/str-deal-search/STR_DSCR_Analysis.xlsx
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="887">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="902">
   <si>
     <t xml:space="preserve">STR DSCR Search: Summary of Top Picks</t>
   </si>
@@ -468,7 +468,7 @@
     <t xml:space="preserve">Monroe</t>
   </si>
   <si>
-    <t xml:space="preserve">Keys: low millage (~1.0-1.2% of price est.). Base ins. = Keys house wind+HO+STR liability; flood by zone on top. Condos use per-row override.</t>
+    <t xml:space="preserve">Keys: ~7.9-9.0 mills (2026) -&gt; 0.70-0.90% of price + $800-1,200/yr non-ad valorem (solid waste, wastewater). Base ins. = wind + non-wind STR policy for an elevated CBS house; flood by zone on top (~$12.5k AE total). Ground-level pre-FIRM: override ~$20k+. Condos: per-row HO-6 override.</t>
   </si>
   <si>
     <t xml:space="preserve">OPERATING PROFILE</t>
@@ -1899,6 +1899,24 @@
     <t xml:space="preserve">Verdict for this buyer</t>
   </si>
   <si>
+    <t xml:space="preserve">KEYS-WIDE 2026 (context)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mixed; verify per parcel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median SFH ~$1.02M, condo ~$610k (Aug 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~6,500 STR listings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balanced-to-buyer-leaning: prices flat (+/-5%), DOM 100-150, ~6.6 months supply (single source); condos favor buyers. Bed tax FY25 $60.8M (-1%); RevPAR ~+10% YTD 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance ($12k+ house) + HOA ($800-2,000 condo) are the DSCR killers</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marathon (city)</t>
   </si>
   <si>
@@ -2848,6 +2866,33 @@
   </si>
   <si>
     <t xml:space="preserve">Visit Florida Keys partner newsletter (Sep 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keys insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OIR county averages (Monroe $7,863 w/ wind, Mar 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citizens STR eligibility (ATB 006-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keys tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FL DOR millage comparison 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keys market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KeysListings market report (Aug 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keys storms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monroe County Irma recovery (1,179 destroyed / 2,977 major)</t>
   </si>
   <si>
     <t xml:space="preserve">Tourism</t>
@@ -3911,15 +3956,15 @@
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$W$7</f>
-        <v>5510.28464609673</v>
+        <v>5390.49297943007</v>
       </c>
       <c r="G12" s="7" t="n">
         <f aca="false">'Monroe (Keys)'!$X$7</f>
-        <v>1.51232356739254</v>
+        <v>1.54593158086525</v>
       </c>
       <c r="H12" s="7" t="n">
         <f aca="false">'Monroe (Keys)'!$Y$7</f>
-        <v>1.20985885391403</v>
+        <v>1.2367452646922</v>
       </c>
       <c r="I12" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$Z$7</f>
@@ -3927,11 +3972,11 @@
       </c>
       <c r="J12" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AD$7</f>
-        <v>-6323.41575316078</v>
+        <v>-4885.91575316079</v>
       </c>
       <c r="K12" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AE$7</f>
-        <v>-26323.4157531608</v>
+        <v>-24885.9157531608</v>
       </c>
       <c r="L12" s="9" t="s">
         <v>25</v>
@@ -3959,15 +4004,15 @@
       </c>
       <c r="F13" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$W$6</f>
-        <v>6076.73812965363</v>
+        <v>5940.07146298696</v>
       </c>
       <c r="G13" s="7" t="n">
         <f aca="false">'Monroe (Keys)'!$X$6</f>
-        <v>1.35736198554988</v>
+        <v>1.38859159939899</v>
       </c>
       <c r="H13" s="7" t="n">
         <f aca="false">'Monroe (Keys)'!$Y$6</f>
-        <v>1.08588958843991</v>
+        <v>1.11087327951919</v>
       </c>
       <c r="I13" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$Z$6</f>
@@ -3975,11 +4020,11 @@
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AD$6</f>
-        <v>-13804.2575558435</v>
+        <v>-12164.2575558435</v>
       </c>
       <c r="K13" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AE$6</f>
-        <v>-33600.2575558435</v>
+        <v>-31960.2575558435</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>26</v>
@@ -4141,12 +4186,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4154,22 +4199,22 @@
         <v>112</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4177,22 +4222,22 @@
         <v>79</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4200,22 +4245,22 @@
         <v>79</v>
       </c>
       <c r="B6" s="48" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D6" s="48" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="F6" s="48" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G6" s="48" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4223,22 +4268,22 @@
         <v>79</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4246,22 +4291,22 @@
         <v>79</v>
       </c>
       <c r="B8" s="48" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="C8" s="48" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="D8" s="48" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="F8" s="48" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="G8" s="48" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4269,22 +4314,22 @@
         <v>79</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4292,22 +4337,22 @@
         <v>81</v>
       </c>
       <c r="B10" s="48" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="C10" s="48" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="D10" s="48" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="E10" s="48" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="F10" s="48" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="G10" s="48" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4315,45 +4360,45 @@
         <v>81</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>415</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="C12" s="48" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="D12" s="48" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="E12" s="48" t="s">
         <v>415</v>
       </c>
       <c r="F12" s="48" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="G12" s="48" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4361,22 +4406,22 @@
         <v>81</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>415</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4384,36 +4429,36 @@
         <v>81</v>
       </c>
       <c r="B14" s="48" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="C14" s="48" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D14" s="48" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="E14" s="48" t="s">
         <v>415</v>
       </c>
       <c r="F14" s="48" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="G14" s="48" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>415</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>415</v>
@@ -4422,7 +4467,7 @@
         <v>415</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4430,22 +4475,22 @@
         <v>18</v>
       </c>
       <c r="B16" s="48" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="C16" s="48" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D16" s="48" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="E16" s="48" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="F16" s="48" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G16" s="48" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4453,22 +4498,22 @@
         <v>18</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4476,22 +4521,22 @@
         <v>18</v>
       </c>
       <c r="B18" s="48" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D18" s="48" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="E18" s="48" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="F18" s="48" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G18" s="48" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4499,22 +4544,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4522,10 +4567,10 @@
         <v>18</v>
       </c>
       <c r="B20" s="48" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="C20" s="48" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="D20" s="48" t="s">
         <v>415</v>
@@ -4534,10 +4579,10 @@
         <v>415</v>
       </c>
       <c r="F20" s="48" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="G20" s="48" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4545,22 +4590,22 @@
         <v>18</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>415</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4568,22 +4613,22 @@
         <v>18</v>
       </c>
       <c r="B22" s="48" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="C22" s="48" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="D22" s="48" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="E22" s="48" t="s">
         <v>415</v>
       </c>
       <c r="F22" s="48" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="G22" s="48" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4591,22 +4636,22 @@
         <v>18</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4614,22 +4659,22 @@
         <v>18</v>
       </c>
       <c r="B24" s="48" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="C24" s="48" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="D24" s="48" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="E24" s="48" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="F24" s="48" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="G24" s="48" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4637,10 +4682,10 @@
         <v>18</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>415</v>
@@ -4649,10 +4694,10 @@
         <v>415</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4660,22 +4705,22 @@
         <v>18</v>
       </c>
       <c r="B26" s="48" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="C26" s="48" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="D26" s="48" t="s">
         <v>415</v>
       </c>
       <c r="E26" s="48" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="F26" s="48" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="G26" s="48" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4683,22 +4728,22 @@
         <v>84</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4706,22 +4751,22 @@
         <v>84</v>
       </c>
       <c r="B28" s="48" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="C28" s="48" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D28" s="48" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="E28" s="48" t="s">
         <v>415</v>
       </c>
       <c r="F28" s="48" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G28" s="48" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4729,22 +4774,22 @@
         <v>84</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>415</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4752,10 +4797,10 @@
         <v>84</v>
       </c>
       <c r="B30" s="48" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="C30" s="48" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="D30" s="48" t="s">
         <v>415</v>
@@ -4764,10 +4809,10 @@
         <v>415</v>
       </c>
       <c r="F30" s="48" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="G30" s="48" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4775,22 +4820,22 @@
         <v>86</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4798,22 +4843,22 @@
         <v>88</v>
       </c>
       <c r="B32" s="48" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="C32" s="48" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D32" s="48" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="E32" s="48" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="F32" s="48" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="G32" s="48" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4821,10 +4866,10 @@
         <v>88</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>415</v>
@@ -4833,21 +4878,21 @@
         <v>415</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="48" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="B34" s="48" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="C34" s="48" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="D34" s="48" t="s">
         <v>415</v>
@@ -4859,7 +4904,7 @@
         <v>526</v>
       </c>
       <c r="G34" s="48" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4867,22 +4912,22 @@
         <v>90</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4890,22 +4935,22 @@
         <v>90</v>
       </c>
       <c r="B36" s="48" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="C36" s="48" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="D36" s="48" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="E36" s="48" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="F36" s="48" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="G36" s="48" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4913,22 +4958,22 @@
         <v>90</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4936,22 +4981,22 @@
         <v>90</v>
       </c>
       <c r="B38" s="48" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="C38" s="48" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="D38" s="48" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="E38" s="48" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="F38" s="48" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="G38" s="48" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4959,22 +5004,22 @@
         <v>90</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>806</v>
+        <v>812</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4982,10 +5027,10 @@
         <v>90</v>
       </c>
       <c r="B40" s="48" t="s">
-        <v>807</v>
+        <v>813</v>
       </c>
       <c r="C40" s="48" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="D40" s="48" t="s">
         <v>415</v>
@@ -4994,10 +5039,10 @@
         <v>415</v>
       </c>
       <c r="F40" s="48" t="s">
-        <v>809</v>
+        <v>815</v>
       </c>
       <c r="G40" s="48" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5005,13 +5050,13 @@
         <v>90</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>415</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>415</v>
@@ -5020,7 +5065,7 @@
         <v>415</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>812</v>
+        <v>818</v>
       </c>
     </row>
   </sheetData>
@@ -5049,23 +5094,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>817</v>
+        <v>823</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5073,10 +5118,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>819</v>
+        <v>825</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5084,10 +5129,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="48" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5095,10 +5140,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>823</v>
+        <v>829</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5106,10 +5151,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="48" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
       <c r="C8" s="48" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5117,10 +5162,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>827</v>
+        <v>833</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5128,10 +5173,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="48" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="C10" s="48" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5139,10 +5184,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5150,10 +5195,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
       <c r="C12" s="48" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5161,10 +5206,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>835</v>
+        <v>841</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5172,10 +5217,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="48" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
       <c r="C14" s="48" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
     </row>
   </sheetData>
@@ -5194,7 +5239,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -5204,23 +5249,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5228,7 +5273,7 @@
         <v>565</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
       <c r="C5" s="33" t="s">
         <v>216</v>
@@ -5239,7 +5284,7 @@
         <v>565</v>
       </c>
       <c r="B6" s="48" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="C6" s="33" t="s">
         <v>216</v>
@@ -5247,10 +5292,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="C7" s="33" t="s">
         <v>216</v>
@@ -5258,10 +5303,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="48" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="B8" s="48" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="C8" s="33" t="s">
         <v>216</v>
@@ -5269,10 +5314,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="C9" s="33" t="s">
         <v>216</v>
@@ -5280,10 +5325,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="48" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B10" s="48" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="C10" s="33" t="s">
         <v>216</v>
@@ -5291,10 +5336,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="C11" s="33" t="s">
         <v>216</v>
@@ -5302,10 +5347,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="C12" s="33" t="s">
         <v>216</v>
@@ -5313,10 +5358,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="C13" s="33" t="s">
         <v>216</v>
@@ -5324,10 +5369,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="48" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="B14" s="48" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="C14" s="33" t="s">
         <v>216</v>
@@ -5335,10 +5380,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="C15" s="33" t="s">
         <v>216</v>
@@ -5346,10 +5391,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="48" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="B16" s="48" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="C16" s="33" t="s">
         <v>216</v>
@@ -5357,10 +5402,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="C17" s="33" t="s">
         <v>216</v>
@@ -5368,10 +5413,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="48" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="B18" s="48" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="C18" s="33" t="s">
         <v>216</v>
@@ -5379,10 +5424,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
       <c r="C19" s="33" t="s">
         <v>216</v>
@@ -5390,10 +5435,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="48" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="B20" s="48" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
       <c r="C20" s="33" t="s">
         <v>216</v>
@@ -5401,10 +5446,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="C21" s="33" t="s">
         <v>216</v>
@@ -5412,10 +5457,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="48" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="B22" s="48" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="C22" s="33" t="s">
         <v>216</v>
@@ -5423,10 +5468,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="C23" s="33" t="s">
         <v>216</v>
@@ -5434,10 +5479,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="48" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="B24" s="48" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="C24" s="33" t="s">
         <v>216</v>
@@ -5445,10 +5490,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="C25" s="33" t="s">
         <v>216</v>
@@ -5456,10 +5501,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="B26" s="48" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="C26" s="33" t="s">
         <v>216</v>
@@ -5467,10 +5512,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="C27" s="33" t="s">
         <v>216</v>
@@ -5478,10 +5523,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="B28" s="48" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="C28" s="33" t="s">
         <v>216</v>
@@ -5489,10 +5534,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="C29" s="33" t="s">
         <v>216</v>
@@ -5500,10 +5545,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="48" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="B30" s="48" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
       <c r="C30" s="33" t="s">
         <v>216</v>
@@ -5511,10 +5556,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="C31" s="33" t="s">
         <v>216</v>
@@ -5522,12 +5567,67 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="48" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
       <c r="B32" s="48" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="C32" s="33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>891</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>893</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="48" t="s">
+        <v>894</v>
+      </c>
+      <c r="B34" s="48" t="s">
+        <v>895</v>
+      </c>
+      <c r="C34" s="33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>896</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>897</v>
+      </c>
+      <c r="C35" s="33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="48" t="s">
+        <v>898</v>
+      </c>
+      <c r="B36" s="48" t="s">
+        <v>899</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>900</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>901</v>
+      </c>
+      <c r="C37" s="33" t="s">
         <v>216</v>
       </c>
     </row>
@@ -5561,6 +5661,11 @@
     <hyperlink ref="C30" r:id="rId26" display="Link"/>
     <hyperlink ref="C31" r:id="rId27" display="Link"/>
     <hyperlink ref="C32" r:id="rId28" display="Link"/>
+    <hyperlink ref="C33" r:id="rId29" display="Link"/>
+    <hyperlink ref="C34" r:id="rId30" display="Link"/>
+    <hyperlink ref="C35" r:id="rId31" display="Link"/>
+    <hyperlink ref="C36" r:id="rId32" display="Link"/>
+    <hyperlink ref="C37" r:id="rId33" display="Link"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5920,15 +6025,15 @@
         <v>89</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="4" t="s">
         <v>90</v>
       </c>
       <c r="C34" s="20" t="n">
-        <v>0.011</v>
+        <v>0.0095</v>
       </c>
       <c r="D34" s="22" t="n">
-        <v>14000</v>
+        <v>8000</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>91</v>
@@ -10399,7 +10504,7 @@
         <v>1200</v>
       </c>
       <c r="P6" s="19" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="Q6" s="27" t="s">
         <v>99</v>
@@ -10418,23 +10523,23 @@
       </c>
       <c r="U6" s="21" t="n">
         <f aca="false">H6*INDEX(Assumptions!$C$28:$C$34,MATCH(D6,Assumptions!$B$28:$B$34,0))/12</f>
-        <v>696.666666666667</v>
+        <v>601.666666666667</v>
       </c>
       <c r="V6" s="21" t="n">
         <f aca="false">IF(ISNUMBER(P6),P6,INDEX(Assumptions!$D$28:$D$34,MATCH(D6,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH(M6,Assumptions!$B$22:$B$25,0)))/12</f>
-        <v>291.666666666667</v>
+        <v>250</v>
       </c>
       <c r="W6" s="21" t="n">
         <f aca="false">T6+U6+V6+O6</f>
-        <v>6076.73812965363</v>
+        <v>5940.07146298696</v>
       </c>
       <c r="X6" s="30" t="n">
         <f aca="false">IFERROR(K6/12/W6,0)</f>
-        <v>1.35736198554988</v>
+        <v>1.38859159939899</v>
       </c>
       <c r="Y6" s="31" t="n">
         <f aca="false">IFERROR(K6*Assumptions!$C$18/12/W6,0)</f>
-        <v>1.08588958843991</v>
+        <v>1.11087327951919</v>
       </c>
       <c r="Z6" s="32" t="n">
         <f aca="false">H6*J6+H6*(Assumptions!$C$16-I6)</f>
@@ -10442,7 +10547,7 @@
       </c>
       <c r="AA6" s="21" t="n">
         <f aca="false">W6*Assumptions!$C$17</f>
-        <v>36460.4287779218</v>
+        <v>35640.4287779218</v>
       </c>
       <c r="AB6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$H$37:$H$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N6="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
@@ -10454,11 +10559,11 @@
       </c>
       <c r="AD6" s="21" t="n">
         <f aca="false">K6-AB6-W6*12</f>
-        <v>-13804.2575558435</v>
+        <v>-12164.2575558435</v>
       </c>
       <c r="AE6" s="21" t="n">
         <f aca="false">AD6-AC6</f>
-        <v>-33600.2575558435</v>
+        <v>-31960.2575558435</v>
       </c>
       <c r="AF6" s="23" t="n">
         <f aca="false">IFERROR(K6/H6,0)</f>
@@ -10525,7 +10630,7 @@
         <v>1448</v>
       </c>
       <c r="P7" s="37" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="Q7" s="36" t="s">
         <v>99</v>
@@ -10544,23 +10649,23 @@
       </c>
       <c r="U7" s="40" t="n">
         <f aca="false">H7*INDEX(Assumptions!$C$28:$C$34,MATCH(D7,Assumptions!$B$28:$B$34,0))/12</f>
-        <v>572.916666666667</v>
+        <v>494.791666666667</v>
       </c>
       <c r="V7" s="40" t="n">
         <f aca="false">IF(ISNUMBER(P7),P7,INDEX(Assumptions!$D$28:$D$34,MATCH(D7,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH(M7,Assumptions!$B$22:$B$25,0)))/12</f>
-        <v>291.666666666667</v>
+        <v>250</v>
       </c>
       <c r="W7" s="40" t="n">
         <f aca="false">T7+U7+V7+O7</f>
-        <v>5510.28464609673</v>
+        <v>5390.49297943007</v>
       </c>
       <c r="X7" s="42" t="n">
         <f aca="false">IFERROR(K7/12/W7,0)</f>
-        <v>1.51232356739254</v>
+        <v>1.54593158086525</v>
       </c>
       <c r="Y7" s="42" t="n">
         <f aca="false">IFERROR(K7*Assumptions!$C$18/12/W7,0)</f>
-        <v>1.20985885391403</v>
+        <v>1.2367452646922</v>
       </c>
       <c r="Z7" s="40" t="n">
         <f aca="false">H7*J7+H7*(Assumptions!$C$16-I7)</f>
@@ -10568,7 +10673,7 @@
       </c>
       <c r="AA7" s="40" t="n">
         <f aca="false">W7*Assumptions!$C$17</f>
-        <v>33061.7078765804</v>
+        <v>32342.9578765804</v>
       </c>
       <c r="AB7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$H$37:$H$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N7="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
@@ -10580,11 +10685,11 @@
       </c>
       <c r="AD7" s="40" t="n">
         <f aca="false">K7-AB7-W7*12</f>
-        <v>-6323.41575316078</v>
+        <v>-4885.91575316079</v>
       </c>
       <c r="AE7" s="40" t="n">
         <f aca="false">AD7-AC7</f>
-        <v>-26323.4157531608</v>
+        <v>-24885.9157531608</v>
       </c>
       <c r="AF7" s="43" t="n">
         <f aca="false">IFERROR(K7/H7,0)</f>
@@ -10653,7 +10758,7 @@
         <v>1448</v>
       </c>
       <c r="P8" s="19" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="Q8" s="27" t="s">
         <v>99</v>
@@ -10672,23 +10777,23 @@
       </c>
       <c r="U8" s="21" t="n">
         <f aca="false">H8*INDEX(Assumptions!$C$28:$C$34,MATCH(D8,Assumptions!$B$28:$B$34,0))/12</f>
-        <v>614.166666666667</v>
+        <v>530.416666666667</v>
       </c>
       <c r="V8" s="21" t="n">
         <f aca="false">IF(ISNUMBER(P8),P8,INDEX(Assumptions!$D$28:$D$34,MATCH(D8,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH(M8,Assumptions!$B$22:$B$25,0)))/12</f>
-        <v>291.666666666667</v>
+        <v>250</v>
       </c>
       <c r="W8" s="21" t="n">
         <f aca="false">T8+U8+V8+O8</f>
-        <v>5781.7691406157</v>
+        <v>5656.35247394903</v>
       </c>
       <c r="X8" s="30" t="n">
         <f aca="false">IFERROR(K8/12/W8,0)</f>
-        <v>0.835788011559856</v>
+        <v>0.854319697294182</v>
       </c>
       <c r="Y8" s="30" t="n">
         <f aca="false">IFERROR(K8*Assumptions!$C$18/12/W8,0)</f>
-        <v>0.668630409247885</v>
+        <v>0.683455757835346</v>
       </c>
       <c r="Z8" s="21" t="n">
         <f aca="false">H8*J8+H8*(Assumptions!$C$16-I8)</f>
@@ -10696,7 +10801,7 @@
       </c>
       <c r="AA8" s="21" t="n">
         <f aca="false">W8*Assumptions!$C$17</f>
-        <v>34690.6148436942</v>
+        <v>33938.1148436942</v>
       </c>
       <c r="AB8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$H$37:$H$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N8="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
@@ -10708,11 +10813,11 @@
       </c>
       <c r="AD8" s="21" t="n">
         <f aca="false">K8-AB8-W8*12</f>
-        <v>-37729.2696873884</v>
+        <v>-36224.2696873884</v>
       </c>
       <c r="AE8" s="21" t="n">
         <f aca="false">AD8-AC8</f>
-        <v>-49326.8696873884</v>
+        <v>-47821.8696873884</v>
       </c>
       <c r="AF8" s="23" t="n">
         <f aca="false">IFERROR(K8/H8,0)</f>
@@ -10779,7 +10884,7 @@
         <v>1448</v>
       </c>
       <c r="P9" s="37" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="Q9" s="36" t="s">
         <v>99</v>
@@ -10798,23 +10903,23 @@
       </c>
       <c r="U9" s="40" t="n">
         <f aca="false">H9*INDEX(Assumptions!$C$28:$C$34,MATCH(D9,Assumptions!$B$28:$B$34,0))/12</f>
-        <v>595.833333333333</v>
+        <v>514.583333333333</v>
       </c>
       <c r="V9" s="40" t="n">
         <f aca="false">IF(ISNUMBER(P9),P9,INDEX(Assumptions!$D$28:$D$34,MATCH(D9,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH(M9,Assumptions!$B$22:$B$25,0)))/12</f>
-        <v>291.666666666667</v>
+        <v>250</v>
       </c>
       <c r="W9" s="40" t="n">
         <f aca="false">T9+U9+V9+O9</f>
-        <v>5661.10936527394</v>
+        <v>5538.19269860727</v>
       </c>
       <c r="X9" s="42" t="n">
         <f aca="false">IFERROR(K9/12/W9,0)</f>
-        <v>0.721295610076197</v>
+        <v>0.737304307659826</v>
       </c>
       <c r="Y9" s="42" t="n">
         <f aca="false">IFERROR(K9*Assumptions!$C$18/12/W9,0)</f>
-        <v>0.577036488060957</v>
+        <v>0.58984344612786</v>
       </c>
       <c r="Z9" s="40" t="n">
         <f aca="false">H9*J9+H9*(Assumptions!$C$16-I9)</f>
@@ -10822,7 +10927,7 @@
       </c>
       <c r="AA9" s="40" t="n">
         <f aca="false">W9*Assumptions!$C$17</f>
-        <v>33966.6561916436</v>
+        <v>33229.1561916436</v>
       </c>
       <c r="AB9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$H$37:$H$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N9="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
@@ -10834,11 +10939,11 @@
       </c>
       <c r="AD9" s="40" t="n">
         <f aca="false">K9-AB9-W9*12</f>
-        <v>-42303.3123832872</v>
+        <v>-40828.3123832872</v>
       </c>
       <c r="AE9" s="40" t="n">
         <f aca="false">AD9-AC9</f>
-        <v>-52103.3123832872</v>
+        <v>-50628.3123832872</v>
       </c>
       <c r="AF9" s="43" t="n">
         <f aca="false">IFERROR(K9/H9,0)</f>
@@ -10905,7 +11010,7 @@
         <v>1404</v>
       </c>
       <c r="P10" s="19" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="Q10" s="27" t="s">
         <v>99</v>
@@ -10924,23 +11029,23 @@
       </c>
       <c r="U10" s="21" t="n">
         <f aca="false">H10*INDEX(Assumptions!$C$28:$C$34,MATCH(D10,Assumptions!$B$28:$B$34,0))/12</f>
-        <v>733.333333333333</v>
+        <v>633.333333333333</v>
       </c>
       <c r="V10" s="21" t="n">
         <f aca="false">IF(ISNUMBER(P10),P10,INDEX(Assumptions!$D$28:$D$34,MATCH(D10,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH(M10,Assumptions!$B$22:$B$25,0)))/12</f>
-        <v>291.666666666667</v>
+        <v>250</v>
       </c>
       <c r="W10" s="21" t="n">
         <f aca="false">T10+U10+V10+O10</f>
-        <v>6522.05768033715</v>
+        <v>6380.39101367049</v>
       </c>
       <c r="X10" s="30" t="n">
         <f aca="false">IFERROR(K10/12/W10,0)</f>
-        <v>1.27771536864153</v>
+        <v>1.30608505269952</v>
       </c>
       <c r="Y10" s="30" t="n">
         <f aca="false">IFERROR(K10*Assumptions!$C$18/12/W10,0)</f>
-        <v>1.02217229491323</v>
+        <v>1.04486804215961</v>
       </c>
       <c r="Z10" s="21" t="n">
         <f aca="false">H10*J10+H10*(Assumptions!$C$16-I10)</f>
@@ -10948,7 +11053,7 @@
       </c>
       <c r="AA10" s="21" t="n">
         <f aca="false">W10*Assumptions!$C$17</f>
-        <v>39132.3460820229</v>
+        <v>38282.3460820229</v>
       </c>
       <c r="AB10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$H$37:$H$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N10="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
@@ -10960,11 +11065,11 @@
       </c>
       <c r="AD10" s="21" t="n">
         <f aca="false">K10-AB10-W10*12</f>
-        <v>-18464.6921640458</v>
+        <v>-16764.6921640458</v>
       </c>
       <c r="AE10" s="21" t="n">
         <f aca="false">AD10-AC10</f>
-        <v>-38464.6921640458</v>
+        <v>-36764.6921640458</v>
       </c>
       <c r="AF10" s="23" t="n">
         <f aca="false">IFERROR(K10/H10,0)</f>
@@ -11033,7 +11138,7 @@
         <v>1448</v>
       </c>
       <c r="P11" s="37" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="Q11" s="36" t="s">
         <v>99</v>
@@ -11052,23 +11157,23 @@
       </c>
       <c r="U11" s="40" t="n">
         <f aca="false">H11*INDEX(Assumptions!$C$28:$C$34,MATCH(D11,Assumptions!$B$28:$B$34,0))/12</f>
-        <v>490.416666666667</v>
+        <v>423.541666666667</v>
       </c>
       <c r="V11" s="40" t="n">
         <f aca="false">IF(ISNUMBER(P11),P11,INDEX(Assumptions!$D$28:$D$34,MATCH(D11,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH(M11,Assumptions!$B$22:$B$25,0)))/12</f>
-        <v>291.666666666667</v>
+        <v>250</v>
       </c>
       <c r="W11" s="40" t="n">
         <f aca="false">T11+U11+V11+O11</f>
-        <v>4967.3156570588</v>
+        <v>4858.77399039214</v>
       </c>
       <c r="X11" s="42" t="n">
         <f aca="false">IFERROR(K11/12/W11,0)</f>
-        <v>0.63750059092111</v>
+        <v>0.651741915332657</v>
       </c>
       <c r="Y11" s="42" t="n">
         <f aca="false">IFERROR(K11*Assumptions!$C$18/12/W11,0)</f>
-        <v>0.510000472736888</v>
+        <v>0.521393532266126</v>
       </c>
       <c r="Z11" s="40" t="n">
         <f aca="false">H11*J11+H11*(Assumptions!$C$16-I11)</f>
@@ -11076,7 +11181,7 @@
       </c>
       <c r="AA11" s="40" t="n">
         <f aca="false">W11*Assumptions!$C$17</f>
-        <v>29803.8939423528</v>
+        <v>29152.6439423528</v>
       </c>
       <c r="AB11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$H$37:$H$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N11="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
@@ -11088,11 +11193,11 @@
       </c>
       <c r="AD11" s="40" t="n">
         <f aca="false">K11-AB11-W11*12</f>
-        <v>-41347.7878847056</v>
+        <v>-40045.2878847056</v>
       </c>
       <c r="AE11" s="40" t="n">
         <f aca="false">AD11-AC11</f>
-        <v>-48947.7878847056</v>
+        <v>-47645.2878847056</v>
       </c>
       <c r="AF11" s="43" t="n">
         <f aca="false">IFERROR(K11/H11,0)</f>
@@ -12427,15 +12532,15 @@
       </c>
       <c r="I25" s="21" t="n">
         <f aca="false">H25+C25*INDEX(Assumptions!$C$28:$C$34,MATCH('Monroe (Keys)'!$D$6,Assumptions!$B$28:$B$34,0))/12+IF(ISNUMBER('Monroe (Keys)'!$P$6),'Monroe (Keys)'!$P$6,INDEX(Assumptions!$D$28:$D$34,MATCH('Monroe (Keys)'!$D$6,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH('Monroe (Keys)'!$M$6,Assumptions!$B$22:$B$25,0)))/12+'Monroe (Keys)'!$O$6</f>
-        <v>6439.55754533423</v>
+        <v>6302.89087866756</v>
       </c>
       <c r="J25" s="30" t="n">
         <f aca="false">IFERROR(E25/12/I25,0)</f>
-        <v>1.28088510355958</v>
+        <v>1.30865875550062</v>
       </c>
       <c r="K25" s="30" t="n">
         <f aca="false">IFERROR(E25*Assumptions!$C$18/12/I25,0)</f>
-        <v>1.02470808284767</v>
+        <v>1.0469270044005</v>
       </c>
       <c r="L25" s="21" t="n">
         <f aca="false">C25*B25+C25*(Assumptions!$C$16-D25)</f>
@@ -12443,15 +12548,15 @@
       </c>
       <c r="M25" s="21" t="n">
         <f aca="false">E25-(E25*INDEX(Assumptions!$H$37:$H$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Monroe (Keys)'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I25*12</f>
-        <v>-18158.0905440108</v>
+        <v>-16518.0905440108</v>
       </c>
       <c r="N25" s="21" t="n">
         <f aca="false">M25-E25*INDEX(Assumptions!$C$37:$C$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-37954.0905440108</v>
+        <v>-36314.0905440108</v>
       </c>
       <c r="O25" s="23" t="n">
         <f aca="false">IFERROR(M25/L25,0)</f>
-        <v>-0.099550935000059</v>
+        <v>-0.0905597069298836</v>
       </c>
       <c r="P25" s="47" t="s">
         <v>415</v>
@@ -12491,15 +12596,15 @@
       </c>
       <c r="I26" s="21" t="n">
         <f aca="false">H26+C26*INDEX(Assumptions!$C$28:$C$34,MATCH('Monroe (Keys)'!$D$6,Assumptions!$B$28:$B$34,0))/12+IF(ISNUMBER('Monroe (Keys)'!$P$6),'Monroe (Keys)'!$P$6,INDEX(Assumptions!$D$28:$D$34,MATCH('Monroe (Keys)'!$D$6,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH('Monroe (Keys)'!$M$6,Assumptions!$B$22:$B$25,0)))/12+'Monroe (Keys)'!$O$6</f>
-        <v>6076.73812965363</v>
+        <v>5940.07146298696</v>
       </c>
       <c r="J26" s="30" t="n">
         <f aca="false">IFERROR(E26/12/I26,0)</f>
-        <v>1.35736198554988</v>
+        <v>1.38859159939899</v>
       </c>
       <c r="K26" s="30" t="n">
         <f aca="false">IFERROR(E26*Assumptions!$C$18/12/I26,0)</f>
-        <v>1.08588958843991</v>
+        <v>1.11087327951919</v>
       </c>
       <c r="L26" s="21" t="n">
         <f aca="false">C26*B26+C26*(Assumptions!$C$16-D26)</f>
@@ -12507,15 +12612,15 @@
       </c>
       <c r="M26" s="21" t="n">
         <f aca="false">E26-(E26*INDEX(Assumptions!$H$37:$H$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Monroe (Keys)'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I26*12</f>
-        <v>-13804.2575558435</v>
+        <v>-12164.2575558435</v>
       </c>
       <c r="N26" s="21" t="n">
         <f aca="false">M26-E26*INDEX(Assumptions!$C$37:$C$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-33600.2575558435</v>
+        <v>-31960.2575558435</v>
       </c>
       <c r="O26" s="23" t="n">
         <f aca="false">IFERROR(M26/L26,0)</f>
-        <v>-0.0626327475310505</v>
+        <v>-0.0551917311971121</v>
       </c>
       <c r="P26" s="23" t="n">
         <f aca="false">IFERROR((M26-M25)/(L26-L25),0)</f>
@@ -12556,15 +12661,15 @@
       </c>
       <c r="I27" s="21" t="n">
         <f aca="false">H27+C27*INDEX(Assumptions!$C$28:$C$34,MATCH('Monroe (Keys)'!$D$6,Assumptions!$B$28:$B$34,0))/12+IF(ISNUMBER('Monroe (Keys)'!$P$6),'Monroe (Keys)'!$P$6,INDEX(Assumptions!$D$28:$D$34,MATCH('Monroe (Keys)'!$D$6,Assumptions!$B$28:$B$34,0))+INDEX(Assumptions!$C$22:$C$25,MATCH('Monroe (Keys)'!$M$6,Assumptions!$B$22:$B$25,0)))/12+'Monroe (Keys)'!$O$6</f>
-        <v>5772.51587729537</v>
+        <v>5635.8492106287</v>
       </c>
       <c r="J27" s="30" t="n">
         <f aca="false">IFERROR(E27/12/I27,0)</f>
-        <v>1.42889747012666</v>
+        <v>1.46354755513645</v>
       </c>
       <c r="K27" s="30" t="n">
         <f aca="false">IFERROR(E27*Assumptions!$C$18/12/I27,0)</f>
-        <v>1.14311797610133</v>
+        <v>1.17083804410916</v>
       </c>
       <c r="L27" s="21" t="n">
         <f aca="false">C27*B27+C27*(Assumptions!$C$16-D27)</f>
@@ -12572,19 +12677,19 @@
       </c>
       <c r="M27" s="21" t="n">
         <f aca="false">E27-(E27*INDEX(Assumptions!$H$37:$H$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Monroe (Keys)'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I27*12</f>
-        <v>-10153.5905275444</v>
+        <v>-8513.59052754439</v>
       </c>
       <c r="N27" s="21" t="n">
         <f aca="false">M27-E27*INDEX(Assumptions!$C$37:$C$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-29949.5905275444</v>
+        <v>-28309.5905275444</v>
       </c>
       <c r="O27" s="23" t="n">
         <f aca="false">IFERROR(M27/L27,0)</f>
-        <v>-0.0392940809889489</v>
+        <v>-0.0329473317629427</v>
       </c>
       <c r="P27" s="23" t="n">
         <f aca="false">IFERROR((M27-M26)/(L27-L26),0)</f>
-        <v>0.0960701849552405</v>
+        <v>0.0960701849552401</v>
       </c>
     </row>
   </sheetData>
@@ -13220,7 +13325,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -13268,7 +13373,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>568</v>
       </c>
@@ -13279,201 +13384,227 @@
         <v>570</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>571</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>572</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>573</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>574</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
+        <v>574</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>575</v>
+      </c>
+      <c r="C6" s="48" t="s">
         <v>576</v>
       </c>
-      <c r="B6" s="48" t="s">
+      <c r="D6" s="48" t="s">
         <v>577</v>
       </c>
-      <c r="C6" s="48" t="s">
+      <c r="E6" s="48" t="s">
         <v>578</v>
       </c>
-      <c r="D6" s="48" t="s">
+      <c r="F6" s="48" t="s">
         <v>579</v>
       </c>
-      <c r="E6" s="48" t="s">
+      <c r="G6" s="48" t="s">
         <v>580</v>
       </c>
-      <c r="F6" s="48" t="s">
+      <c r="H6" s="48" t="s">
         <v>581</v>
-      </c>
-      <c r="G6" s="48" t="s">
-        <v>582</v>
-      </c>
-      <c r="H6" s="48" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
+        <v>582</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>583</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>584</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>585</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>586</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>587</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>588</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>589</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>590</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>591</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="48" t="s">
+        <v>590</v>
+      </c>
+      <c r="B8" s="48" t="s">
+        <v>591</v>
+      </c>
+      <c r="C8" s="48" t="s">
         <v>592</v>
       </c>
-      <c r="B8" s="48" t="s">
+      <c r="D8" s="48" t="s">
         <v>593</v>
       </c>
-      <c r="C8" s="48" t="s">
+      <c r="E8" s="48" t="s">
         <v>594</v>
       </c>
-      <c r="D8" s="48" t="s">
+      <c r="F8" s="48" t="s">
         <v>595</v>
       </c>
-      <c r="E8" s="48" t="s">
+      <c r="G8" s="48" t="s">
         <v>596</v>
       </c>
-      <c r="F8" s="48" t="s">
+      <c r="H8" s="48" t="s">
         <v>597</v>
       </c>
-      <c r="G8" s="48" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
         <v>598</v>
       </c>
-      <c r="H8" s="48" t="s">
+      <c r="B9" s="9" t="s">
         <v>599</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>600</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>601</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="E9" s="9" t="s">
         <v>602</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>603</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="G9" s="9" t="s">
         <v>604</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>605</v>
       </c>
-      <c r="G9" s="9" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="48" t="s">
         <v>606</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="B10" s="48" t="s">
         <v>607</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="48" t="s">
+      <c r="C10" s="48" t="s">
         <v>608</v>
       </c>
-      <c r="B10" s="48" t="s">
+      <c r="D10" s="48" t="s">
         <v>609</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="E10" s="48" t="s">
         <v>610</v>
       </c>
-      <c r="D10" s="48" t="s">
+      <c r="F10" s="48" t="s">
         <v>611</v>
       </c>
-      <c r="E10" s="48" t="s">
+      <c r="G10" s="48" t="s">
         <v>612</v>
       </c>
-      <c r="F10" s="48" t="s">
+      <c r="H10" s="48" t="s">
         <v>613</v>
       </c>
-      <c r="G10" s="48" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
         <v>614</v>
       </c>
-      <c r="H10" s="48" t="s">
+      <c r="B11" s="9" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+      <c r="C11" s="9" t="s">
         <v>616</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="D11" s="9" t="s">
         <v>617</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="E11" s="9" t="s">
         <v>618</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>619</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="G11" s="9" t="s">
         <v>620</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>621</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>622</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>623</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="48" t="s">
+        <v>622</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>623</v>
+      </c>
+      <c r="C12" s="48" t="s">
         <v>624</v>
       </c>
-      <c r="B12" s="48" t="s">
+      <c r="D12" s="48" t="s">
         <v>625</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="E12" s="48" t="s">
         <v>626</v>
       </c>
-      <c r="D12" s="48" t="s">
+      <c r="F12" s="48" t="s">
         <v>627</v>
       </c>
-      <c r="E12" s="48" t="s">
+      <c r="G12" s="48" t="s">
         <v>628</v>
       </c>
-      <c r="F12" s="48" t="s">
+      <c r="H12" s="48" t="s">
         <v>629</v>
       </c>
-      <c r="G12" s="48" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
         <v>630</v>
       </c>
-      <c r="H12" s="48" t="s">
+      <c r="B13" s="9" t="s">
         <v>631</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>633</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>635</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>636</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Model: drop cleaning as an operating cost (passed through to guests)
Cleaning set to 0% in the STR and Seasonal profiles (workbook Assumptions and
dscr_model.py). Gross must exclude guest-paid cleaning fees. #1 cash flow at
25% down moves from -$3.8k to +$4.7k/yr self-managed, -$20.8k to -$12.3k
with full-service PM. Report and Summary notes updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUSnEuGCzSgy6aeiGVU1U4
</commit_message>
<xml_diff>
--- a/str-deal-search/STR_DSCR_Analysis.xlsx
+++ b/str-deal-search/STR_DSCR_Analysis.xlsx
@@ -502,7 +502,7 @@
     <t xml:space="preserve">STR</t>
   </si>
   <si>
-    <t xml:space="preserve">Nightly/weekly. Full-service PM 18-30% locally; Airbnb host-only fee 15.5% (blended 10%); cleaning ~10% of gross (offset if guest-paid fees are inside the seller's gross).</t>
+    <t xml:space="preserve">Nightly/weekly. Full-service PM 18-30% locally; Airbnb host-only fee 15.5% (blended 10%); cleaning = 0: passed through to guests as a cleaning fee. Use gross EXCLUDING guest-paid cleaning fees.</t>
   </si>
   <si>
     <t xml:space="preserve">Seasonal</t>
@@ -5298,11 +5298,11 @@
       </c>
       <c r="J5" s="6" t="n">
         <f aca="false">'Manatee-Sarasota'!$AD$6</f>
-        <v>-3831.68451483207</v>
+        <v>4668.31548516793</v>
       </c>
       <c r="K5" s="6" t="n">
         <f aca="false">'Manatee-Sarasota'!$AE$6</f>
-        <v>-20831.6845148321</v>
+        <v>-12331.6845148321</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>15</v>
@@ -5346,11 +5346,11 @@
       </c>
       <c r="J6" s="6" t="n">
         <f aca="false">'Manatee-Sarasota'!$AD$7</f>
-        <v>-2432.09799432634</v>
+        <v>4867.90200567366</v>
       </c>
       <c r="K6" s="6" t="n">
         <f aca="false">'Manatee-Sarasota'!$AE$7</f>
-        <v>-17032.0979943263</v>
+        <v>-9732.09799432635</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>16</v>
@@ -5394,11 +5394,11 @@
       </c>
       <c r="J7" s="6" t="n">
         <f aca="false">'Manatee-Sarasota'!$AD$8</f>
-        <v>-4207.51912303436</v>
+        <v>4692.48087696564</v>
       </c>
       <c r="K7" s="6" t="n">
         <f aca="false">'Manatee-Sarasota'!$AE$8</f>
-        <v>-22007.5191230344</v>
+        <v>-13107.5191230344</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>17</v>
@@ -5442,11 +5442,11 @@
       </c>
       <c r="J8" s="6" t="n">
         <f aca="false">Pinellas!$AD$6</f>
-        <v>-7966.99462445278</v>
+        <v>-866.994624452775</v>
       </c>
       <c r="K8" s="6" t="n">
         <f aca="false">Pinellas!$AE$6</f>
-        <v>-22166.9946244528</v>
+        <v>-15066.9946244528</v>
       </c>
       <c r="L8" s="9" t="s">
         <v>19</v>
@@ -5490,11 +5490,11 @@
       </c>
       <c r="J9" s="6" t="n">
         <f aca="false">Pinellas!$AD$7</f>
-        <v>1413.00537554723</v>
+        <v>9913.00537554723</v>
       </c>
       <c r="K9" s="6" t="n">
         <f aca="false">Pinellas!$AE$7</f>
-        <v>-15586.9946244528</v>
+        <v>-7086.99462445278</v>
       </c>
       <c r="L9" s="9" t="s">
         <v>20</v>
@@ -5538,11 +5538,11 @@
       </c>
       <c r="J10" s="6" t="n">
         <f aca="false">Pinellas!$AD$8</f>
-        <v>-8344.59416971947</v>
+        <v>-3244.59416971947</v>
       </c>
       <c r="K10" s="6" t="n">
         <f aca="false">Pinellas!$AE$8</f>
-        <v>-18544.5941697195</v>
+        <v>-13444.5941697195</v>
       </c>
       <c r="L10" s="9" t="s">
         <v>21</v>
@@ -5586,11 +5586,11 @@
       </c>
       <c r="J11" s="6" t="n">
         <f aca="false">'Other SWFL Listings'!$AD$6</f>
-        <v>-13862.0979943264</v>
+        <v>-7862.09799432635</v>
       </c>
       <c r="K11" s="6" t="n">
         <f aca="false">'Other SWFL Listings'!$AE$6</f>
-        <v>-25862.0979943264</v>
+        <v>-19862.0979943264</v>
       </c>
       <c r="L11" s="9" t="s">
         <v>23</v>
@@ -5634,11 +5634,11 @@
       </c>
       <c r="J12" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AD$7</f>
-        <v>-4885.91575316079</v>
+        <v>5114.08424683921</v>
       </c>
       <c r="K12" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AE$7</f>
-        <v>-24885.9157531608</v>
+        <v>-14885.9157531608</v>
       </c>
       <c r="L12" s="9" t="s">
         <v>25</v>
@@ -5682,11 +5682,11 @@
       </c>
       <c r="J13" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AD$6</f>
-        <v>-12164.2575558435</v>
+        <v>-2266.25755584351</v>
       </c>
       <c r="K13" s="6" t="n">
         <f aca="false">'Monroe (Keys)'!$AE$6</f>
-        <v>-31960.2575558435</v>
+        <v>-22062.2575558435</v>
       </c>
       <c r="L13" s="9" t="s">
         <v>26</v>
@@ -8054,7 +8054,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="4" t="s">
         <v>100</v>
       </c>
@@ -8065,7 +8065,7 @@
         <v>0.1</v>
       </c>
       <c r="E37" s="18" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
         <v>0.08</v>
@@ -8075,7 +8075,7 @@
       </c>
       <c r="H37" s="23" t="n">
         <f aca="false">SUM(D37:G37)</f>
-        <v>0.33</v>
+        <v>0.23</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>101</v>
@@ -8092,7 +8092,7 @@
         <v>0.02</v>
       </c>
       <c r="E38" s="18" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>0.06</v>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="H38" s="23" t="n">
         <f aca="false">SUM(D38:G38)</f>
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>103</v>
@@ -8423,7 +8423,7 @@
       </c>
       <c r="AB6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$H$37:$H$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N6="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>37050</v>
+        <v>28550</v>
       </c>
       <c r="AC6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$C$37:$C$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))</f>
@@ -8431,11 +8431,11 @@
       </c>
       <c r="AD6" s="21" t="n">
         <f aca="false">K6-AB6-W6*12</f>
-        <v>-3831.68451483207</v>
+        <v>4668.31548516793</v>
       </c>
       <c r="AE6" s="21" t="n">
         <f aca="false">AD6-AC6</f>
-        <v>-20831.6845148321</v>
+        <v>-12331.6845148321</v>
       </c>
       <c r="AF6" s="23" t="n">
         <f aca="false">IFERROR(K6/H6,0)</f>
@@ -8443,7 +8443,7 @@
       </c>
       <c r="AG6" s="23" t="n">
         <f aca="false">IFERROR((K6-AB6-AC6)/H6,0)</f>
-        <v>0.0552678571428571</v>
+        <v>0.0704464285714286</v>
       </c>
       <c r="AH6" s="26" t="s">
         <v>146</v>
@@ -8551,7 +8551,7 @@
       </c>
       <c r="AB7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$H$37:$H$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N7="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>31290</v>
+        <v>23990</v>
       </c>
       <c r="AC7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$C$37:$C$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))</f>
@@ -8559,11 +8559,11 @@
       </c>
       <c r="AD7" s="40" t="n">
         <f aca="false">K7-AB7-W7*12</f>
-        <v>-2432.09799432634</v>
+        <v>4867.90200567366</v>
       </c>
       <c r="AE7" s="40" t="n">
         <f aca="false">AD7-AC7</f>
-        <v>-17032.0979943263</v>
+        <v>-9732.09799432635</v>
       </c>
       <c r="AF7" s="43" t="n">
         <f aca="false">IFERROR(K7/H7,0)</f>
@@ -8571,7 +8571,7 @@
       </c>
       <c r="AG7" s="43" t="n">
         <f aca="false">IFERROR((K7-AB7-AC7)/H7,0)</f>
-        <v>0.0589347826086957</v>
+        <v>0.074804347826087</v>
       </c>
       <c r="AH7" s="35" t="s">
         <v>155</v>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="AB8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$H$37:$H$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N8="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>38370</v>
+        <v>29470</v>
       </c>
       <c r="AC8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$C$37:$C$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))</f>
@@ -8687,11 +8687,11 @@
       </c>
       <c r="AD8" s="21" t="n">
         <f aca="false">K8-AB8-W8*12</f>
-        <v>-4207.51912303436</v>
+        <v>4692.48087696564</v>
       </c>
       <c r="AE8" s="21" t="n">
         <f aca="false">AD8-AC8</f>
-        <v>-22007.5191230344</v>
+        <v>-13107.5191230344</v>
       </c>
       <c r="AF8" s="23" t="n">
         <f aca="false">IFERROR(K8/H8,0)</f>
@@ -8699,7 +8699,7 @@
       </c>
       <c r="AG8" s="23" t="n">
         <f aca="false">IFERROR((K8-AB8-AC8)/H8,0)</f>
-        <v>0.0547166666666667</v>
+        <v>0.06955</v>
       </c>
       <c r="AH8" s="26" t="s">
         <v>161</v>
@@ -8807,7 +8807,7 @@
       </c>
       <c r="AB9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$H$37:$H$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N9="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>27000</v>
+        <v>21000</v>
       </c>
       <c r="AC9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$C$37:$C$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))</f>
@@ -8815,11 +8815,11 @@
       </c>
       <c r="AD9" s="40" t="n">
         <f aca="false">K9-AB9-W9*12</f>
-        <v>-9077.61866830105</v>
+        <v>-3077.61866830105</v>
       </c>
       <c r="AE9" s="40" t="n">
         <f aca="false">AD9-AC9</f>
-        <v>-21077.6186683011</v>
+        <v>-15077.6186683011</v>
       </c>
       <c r="AF9" s="43" t="n">
         <f aca="false">IFERROR(K9/H9,0)</f>
@@ -8827,7 +8827,7 @@
       </c>
       <c r="AG9" s="43" t="n">
         <f aca="false">IFERROR((K9-AB9-AC9)/H9,0)</f>
-        <v>0.0461538461538462</v>
+        <v>0.0593406593406593</v>
       </c>
       <c r="AH9" s="35" t="s">
         <v>167</v>
@@ -8935,7 +8935,7 @@
       </c>
       <c r="AB10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$H$37:$H$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N10="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>26820</v>
+        <v>21420</v>
       </c>
       <c r="AC10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$C$37:$C$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))</f>
@@ -8943,11 +8943,11 @@
       </c>
       <c r="AD10" s="21" t="n">
         <f aca="false">K10-AB10-W10*12</f>
-        <v>-17107.959576537</v>
+        <v>-11707.959576537</v>
       </c>
       <c r="AE10" s="21" t="n">
         <f aca="false">AD10-AC10</f>
-        <v>-27907.959576537</v>
+        <v>-22507.959576537</v>
       </c>
       <c r="AF10" s="23" t="n">
         <f aca="false">IFERROR(K10/H10,0)</f>
@@ -8955,7 +8955,7 @@
       </c>
       <c r="AG10" s="23" t="n">
         <f aca="false">IFERROR((K10-AB10-AC10)/H10,0)</f>
-        <v>0.0344842831248066</v>
+        <v>0.0458527281110066</v>
       </c>
       <c r="AH10" s="26" t="s">
         <v>172</v>
@@ -9063,7 +9063,7 @@
       </c>
       <c r="AB11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$H$37:$H$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N11="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>28800</v>
+        <v>22800</v>
       </c>
       <c r="AC11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$C$37:$C$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))</f>
@@ -9071,11 +9071,11 @@
       </c>
       <c r="AD11" s="40" t="n">
         <f aca="false">K11-AB11-W11*12</f>
-        <v>-17143.8705806045</v>
+        <v>-11143.8705806045</v>
       </c>
       <c r="AE11" s="40" t="n">
         <f aca="false">AD11-AC11</f>
-        <v>-29143.8705806045</v>
+        <v>-23143.8705806045</v>
       </c>
       <c r="AF11" s="43" t="n">
         <f aca="false">IFERROR(K11/H11,0)</f>
@@ -9083,7 +9083,7 @@
       </c>
       <c r="AG11" s="43" t="n">
         <f aca="false">IFERROR((K11-AB11-AC11)/H11,0)</f>
-        <v>0.0372815533980583</v>
+        <v>0.0489320388349515</v>
       </c>
       <c r="AH11" s="35" t="s">
         <v>177</v>
@@ -9191,7 +9191,7 @@
       </c>
       <c r="AB12" s="21" t="n">
         <f aca="false">K12*INDEX(Assumptions!$H$37:$H$38,MATCH(Q12,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N12="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>23751.81</v>
+        <v>18736.11</v>
       </c>
       <c r="AC12" s="21" t="n">
         <f aca="false">K12*INDEX(Assumptions!$C$37:$C$38,MATCH(Q12,Assumptions!$B$37:$B$38,0))</f>
@@ -9199,11 +9199,11 @@
       </c>
       <c r="AD12" s="21" t="n">
         <f aca="false">K12-AB12-W12*12</f>
-        <v>-19417.2219285539</v>
+        <v>-14401.5219285539</v>
       </c>
       <c r="AE12" s="21" t="n">
         <f aca="false">AD12-AC12</f>
-        <v>-29448.6219285539</v>
+        <v>-24432.9219285539</v>
       </c>
       <c r="AF12" s="23" t="n">
         <f aca="false">IFERROR(K12/H12,0)</f>
@@ -9211,7 +9211,7 @@
       </c>
       <c r="AG12" s="23" t="n">
         <f aca="false">IFERROR((K12-AB12-AC12)/H12,0)</f>
-        <v>0.0324233465346535</v>
+        <v>0.0423554257425743</v>
       </c>
       <c r="AH12" s="26" t="s">
         <v>182</v>
@@ -9319,7 +9319,7 @@
       </c>
       <c r="AB13" s="40" t="n">
         <f aca="false">K13*INDEX(Assumptions!$H$37:$H$38,MATCH(Q13,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N13="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>24840</v>
+        <v>20040</v>
       </c>
       <c r="AC13" s="40" t="n">
         <f aca="false">K13*INDEX(Assumptions!$C$37:$C$38,MATCH(Q13,Assumptions!$B$37:$B$38,0))</f>
@@ -9327,11 +9327,11 @@
       </c>
       <c r="AD13" s="40" t="n">
         <f aca="false">K13-AB13-W13*12</f>
-        <v>-26425.8085586803</v>
+        <v>-21625.8085586803</v>
       </c>
       <c r="AE13" s="40" t="n">
         <f aca="false">AD13-AC13</f>
-        <v>-36025.8085586803</v>
+        <v>-31225.8085586803</v>
       </c>
       <c r="AF13" s="43" t="n">
         <f aca="false">IFERROR(K13/H13,0)</f>
@@ -9339,7 +9339,7 @@
       </c>
       <c r="AG13" s="43" t="n">
         <f aca="false">IFERROR((K13-AB13-AC13)/H13,0)</f>
-        <v>0.0255849056603774</v>
+        <v>0.0346415094339623</v>
       </c>
       <c r="AH13" s="35" t="s">
         <v>187</v>
@@ -9447,7 +9447,7 @@
       </c>
       <c r="AB14" s="21" t="n">
         <f aca="false">K14*INDEX(Assumptions!$H$37:$H$38,MATCH(Q14,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N14="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>20400</v>
+        <v>16400</v>
       </c>
       <c r="AC14" s="21" t="n">
         <f aca="false">K14*INDEX(Assumptions!$C$37:$C$38,MATCH(Q14,Assumptions!$B$37:$B$38,0))</f>
@@ -9455,11 +9455,11 @@
       </c>
       <c r="AD14" s="21" t="n">
         <f aca="false">K14-AB14-W14*12</f>
-        <v>-15902.5114738206</v>
+        <v>-11902.5114738206</v>
       </c>
       <c r="AE14" s="21" t="n">
         <f aca="false">AD14-AC14</f>
-        <v>-23902.5114738206</v>
+        <v>-19902.5114738206</v>
       </c>
       <c r="AF14" s="23" t="n">
         <f aca="false">IFERROR(K14/H14,0)</f>
@@ -9467,7 +9467,7 @@
       </c>
       <c r="AG14" s="23" t="n">
         <f aca="false">IFERROR((K14-AB14-AC14)/H14,0)</f>
-        <v>0.0322222222222222</v>
+        <v>0.0433333333333333</v>
       </c>
       <c r="AH14" s="26" t="s">
         <v>192</v>
@@ -9575,7 +9575,7 @@
       </c>
       <c r="AB15" s="40" t="n">
         <f aca="false">K15*INDEX(Assumptions!$H$37:$H$38,MATCH(Q15,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N15="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>23520</v>
+        <v>20460</v>
       </c>
       <c r="AC15" s="40" t="n">
         <f aca="false">K15*INDEX(Assumptions!$C$37:$C$38,MATCH(Q15,Assumptions!$B$37:$B$38,0))</f>
@@ -9583,11 +9583,11 @@
       </c>
       <c r="AD15" s="40" t="n">
         <f aca="false">K15-AB15-W15*12</f>
-        <v>20423.2082906875</v>
+        <v>23483.2082906875</v>
       </c>
       <c r="AE15" s="40" t="n">
         <f aca="false">AD15-AC15</f>
-        <v>8183.20829068749</v>
+        <v>11243.2082906875</v>
       </c>
       <c r="AF15" s="43" t="n">
         <f aca="false">IFERROR(K15/H15,0)</f>
@@ -9595,7 +9595,7 @@
       </c>
       <c r="AG15" s="43" t="n">
         <f aca="false">IFERROR((K15-AB15-AC15)/H15,0)</f>
-        <v>0.101129770992366</v>
+        <v>0.105801526717557</v>
       </c>
       <c r="AH15" s="35" t="s">
         <v>199</v>
@@ -9703,7 +9703,7 @@
       </c>
       <c r="AB16" s="21" t="n">
         <f aca="false">K16*INDEX(Assumptions!$H$37:$H$38,MATCH(Q16,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N16="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>21720</v>
+        <v>17320</v>
       </c>
       <c r="AC16" s="21" t="n">
         <f aca="false">K16*INDEX(Assumptions!$C$37:$C$38,MATCH(Q16,Assumptions!$B$37:$B$38,0))</f>
@@ -9711,11 +9711,11 @@
       </c>
       <c r="AD16" s="21" t="n">
         <f aca="false">K16-AB16-W16*12</f>
-        <v>-13758.446392211</v>
+        <v>-9358.44639221097</v>
       </c>
       <c r="AE16" s="21" t="n">
         <f aca="false">AD16-AC16</f>
-        <v>-22558.446392211</v>
+        <v>-18158.446392211</v>
       </c>
       <c r="AF16" s="23" t="n">
         <f aca="false">IFERROR(K16/H16,0)</f>
@@ -9723,7 +9723,7 @@
       </c>
       <c r="AG16" s="23" t="n">
         <f aca="false">IFERROR((K16-AB16-AC16)/H16,0)</f>
-        <v>0.0483154121863799</v>
+        <v>0.0640860215053763</v>
       </c>
       <c r="AH16" s="26"/>
       <c r="AI16" s="13" t="n">
@@ -9829,7 +9829,7 @@
       </c>
       <c r="AB17" s="40" t="n">
         <f aca="false">K17*INDEX(Assumptions!$H$37:$H$38,MATCH(Q17,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N17="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>23700</v>
+        <v>18700</v>
       </c>
       <c r="AC17" s="40" t="n">
         <f aca="false">K17*INDEX(Assumptions!$C$37:$C$38,MATCH(Q17,Assumptions!$B$37:$B$38,0))</f>
@@ -9837,11 +9837,11 @@
       </c>
       <c r="AD17" s="40" t="n">
         <f aca="false">K17-AB17-W17*12</f>
-        <v>-44398.4578660316</v>
+        <v>-39398.4578660316</v>
       </c>
       <c r="AE17" s="40" t="n">
         <f aca="false">AD17-AC17</f>
-        <v>-54398.4578660316</v>
+        <v>-49398.4578660316</v>
       </c>
       <c r="AF17" s="43" t="n">
         <f aca="false">IFERROR(K17/H17,0)</f>
@@ -9849,7 +9849,7 @@
       </c>
       <c r="AG17" s="43" t="n">
         <f aca="false">IFERROR((K17-AB17-AC17)/H17,0)</f>
-        <v>0.025508607198748</v>
+        <v>0.0333333333333333</v>
       </c>
       <c r="AH17" s="35"/>
       <c r="AI17" s="34" t="n">
@@ -10338,7 +10338,7 @@
       </c>
       <c r="AB6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$H$37:$H$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N6="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>32430</v>
+        <v>25330</v>
       </c>
       <c r="AC6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$C$37:$C$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))</f>
@@ -10346,11 +10346,11 @@
       </c>
       <c r="AD6" s="21" t="n">
         <f aca="false">K6-AB6-W6*12</f>
-        <v>-7966.99462445278</v>
+        <v>-866.994624452775</v>
       </c>
       <c r="AE6" s="21" t="n">
         <f aca="false">AD6-AC6</f>
-        <v>-22166.9946244528</v>
+        <v>-15066.9946244528</v>
       </c>
       <c r="AF6" s="23" t="n">
         <f aca="false">IFERROR(K6/H6,0)</f>
@@ -10358,7 +10358,7 @@
       </c>
       <c r="AG6" s="23" t="n">
         <f aca="false">IFERROR((K6-AB6-AC6)/H6,0)</f>
-        <v>0.0502474226804124</v>
+        <v>0.0648865979381443</v>
       </c>
       <c r="AH6" s="26"/>
       <c r="AI6" s="13" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="AB7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$H$37:$H$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N7="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>37050</v>
+        <v>28550</v>
       </c>
       <c r="AC7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$C$37:$C$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))</f>
@@ -10472,11 +10472,11 @@
       </c>
       <c r="AD7" s="40" t="n">
         <f aca="false">K7-AB7-W7*12</f>
-        <v>1413.00537554723</v>
+        <v>9913.00537554723</v>
       </c>
       <c r="AE7" s="40" t="n">
         <f aca="false">AD7-AC7</f>
-        <v>-15586.9946244528</v>
+        <v>-7086.99462445278</v>
       </c>
       <c r="AF7" s="43" t="n">
         <f aca="false">IFERROR(K7/H7,0)</f>
@@ -10484,7 +10484,7 @@
       </c>
       <c r="AG7" s="43" t="n">
         <f aca="false">IFERROR((K7-AB7-AC7)/H7,0)</f>
-        <v>0.0638144329896907</v>
+        <v>0.081340206185567</v>
       </c>
       <c r="AH7" s="35"/>
       <c r="AI7" s="34" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="AB8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$H$37:$H$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N8="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>24030</v>
+        <v>18930</v>
       </c>
       <c r="AC8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$C$37:$C$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))</f>
@@ -10598,11 +10598,11 @@
       </c>
       <c r="AD8" s="21" t="n">
         <f aca="false">K8-AB8-W8*12</f>
-        <v>-8344.59416971947</v>
+        <v>-3244.59416971947</v>
       </c>
       <c r="AE8" s="21" t="n">
         <f aca="false">AD8-AC8</f>
-        <v>-18544.5941697195</v>
+        <v>-13444.5941697195</v>
       </c>
       <c r="AF8" s="23" t="n">
         <f aca="false">IFERROR(K8/H8,0)</f>
@@ -10610,7 +10610,7 @@
       </c>
       <c r="AG8" s="23" t="n">
         <f aca="false">IFERROR((K8-AB8-AC8)/H8,0)</f>
-        <v>0.0493235294117647</v>
+        <v>0.0643235294117647</v>
       </c>
       <c r="AH8" s="26"/>
       <c r="AI8" s="13" t="n">
@@ -10716,7 +10716,7 @@
       </c>
       <c r="AB9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$H$37:$H$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N9="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>31950</v>
+        <v>24450</v>
       </c>
       <c r="AC9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$C$37:$C$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))</f>
@@ -10724,11 +10724,11 @@
       </c>
       <c r="AD9" s="40" t="n">
         <f aca="false">K9-AB9-W9*12</f>
-        <v>-29515.3537312367</v>
+        <v>-22015.3537312367</v>
       </c>
       <c r="AE9" s="40" t="n">
         <f aca="false">AD9-AC9</f>
-        <v>-44515.3537312367</v>
+        <v>-37015.3537312367</v>
       </c>
       <c r="AF9" s="43" t="n">
         <f aca="false">IFERROR(K9/H9,0)</f>
@@ -10736,7 +10736,7 @@
       </c>
       <c r="AG9" s="43" t="n">
         <f aca="false">IFERROR((K9-AB9-AC9)/H9,0)</f>
-        <v>0.043828125</v>
+        <v>0.055546875</v>
       </c>
       <c r="AH9" s="35"/>
       <c r="AI9" s="34" t="n">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="AB10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$H$37:$H$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N10="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>26670</v>
+        <v>20770</v>
       </c>
       <c r="AC10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$C$37:$C$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))</f>
@@ -10850,11 +10850,11 @@
       </c>
       <c r="AD10" s="21" t="n">
         <f aca="false">K10-AB10-W10*12</f>
-        <v>-30071.6845148321</v>
+        <v>-24171.6845148321</v>
       </c>
       <c r="AE10" s="21" t="n">
         <f aca="false">AD10-AC10</f>
-        <v>-41871.6845148321</v>
+        <v>-35971.6845148321</v>
       </c>
       <c r="AF10" s="23" t="n">
         <f aca="false">IFERROR(K10/H10,0)</f>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="AG10" s="23" t="n">
         <f aca="false">IFERROR((K10-AB10-AC10)/H10,0)</f>
-        <v>0.0366607142857143</v>
+        <v>0.0471964285714286</v>
       </c>
       <c r="AH10" s="26"/>
       <c r="AI10" s="13" t="n">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="AB11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$H$37:$H$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N11="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>14862.4</v>
+        <v>13425.7</v>
       </c>
       <c r="AC11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$C$37:$C$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))</f>
@@ -10976,11 +10976,11 @@
       </c>
       <c r="AD11" s="40" t="n">
         <f aca="false">K11-AB11-W11*12</f>
-        <v>-38655.9604709838</v>
+        <v>-37219.2604709838</v>
       </c>
       <c r="AE11" s="40" t="n">
         <f aca="false">AD11-AC11</f>
-        <v>-44402.7604709838</v>
+        <v>-42966.0604709838</v>
       </c>
       <c r="AF11" s="43" t="n">
         <f aca="false">IFERROR(K11/H11,0)</f>
@@ -10988,7 +10988,7 @@
       </c>
       <c r="AG11" s="43" t="n">
         <f aca="false">IFERROR((K11-AB11-AC11)/H11,0)</f>
-        <v>0.0462386440677966</v>
+        <v>0.0486737288135593</v>
       </c>
       <c r="AH11" s="35"/>
       <c r="AI11" s="34" t="n">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="AB12" s="21" t="n">
         <f aca="false">K12*INDEX(Assumptions!$H$37:$H$38,MATCH(Q12,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N12="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>23700</v>
+        <v>18700</v>
       </c>
       <c r="AC12" s="21" t="n">
         <f aca="false">K12*INDEX(Assumptions!$C$37:$C$38,MATCH(Q12,Assumptions!$B$37:$B$38,0))</f>
@@ -11102,11 +11102,11 @@
       </c>
       <c r="AD12" s="21" t="n">
         <f aca="false">K12-AB12-W12*12</f>
-        <v>-55199.709778335</v>
+        <v>-50199.709778335</v>
       </c>
       <c r="AE12" s="21" t="n">
         <f aca="false">AD12-AC12</f>
-        <v>-65199.709778335</v>
+        <v>-60199.709778335</v>
       </c>
       <c r="AF12" s="23" t="n">
         <f aca="false">IFERROR(K12/H12,0)</f>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="AG12" s="23" t="n">
         <f aca="false">IFERROR((K12-AB12-AC12)/H12,0)</f>
-        <v>0.0233190271816881</v>
+        <v>0.0304721030042918</v>
       </c>
       <c r="AH12" s="26"/>
       <c r="AI12" s="13" t="n">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="AB6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$H$37:$H$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N6="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>28800</v>
+        <v>22800</v>
       </c>
       <c r="AC6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$C$37:$C$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))</f>
@@ -11753,11 +11753,11 @@
       </c>
       <c r="AD6" s="21" t="n">
         <f aca="false">K6-AB6-W6*12</f>
-        <v>-13862.0979943264</v>
+        <v>-7862.09799432635</v>
       </c>
       <c r="AE6" s="21" t="n">
         <f aca="false">AD6-AC6</f>
-        <v>-25862.0979943264</v>
+        <v>-19862.0979943264</v>
       </c>
       <c r="AF6" s="23" t="n">
         <f aca="false">IFERROR(K6/H6,0)</f>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="AG6" s="23" t="n">
         <f aca="false">IFERROR((K6-AB6-AC6)/H6,0)</f>
-        <v>0.0417391304347826</v>
+        <v>0.0547826086956522</v>
       </c>
       <c r="AH6" s="26"/>
       <c r="AI6" s="13" t="n">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="AB7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$H$37:$H$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N7="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>27000</v>
+        <v>21000</v>
       </c>
       <c r="AC7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$C$37:$C$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))</f>
@@ -11879,11 +11879,11 @@
       </c>
       <c r="AD7" s="40" t="n">
         <f aca="false">K7-AB7-W7*12</f>
-        <v>-31741.7208844633</v>
+        <v>-25741.7208844633</v>
       </c>
       <c r="AE7" s="40" t="n">
         <f aca="false">AD7-AC7</f>
-        <v>-43741.7208844633</v>
+        <v>-37741.7208844633</v>
       </c>
       <c r="AF7" s="43" t="n">
         <f aca="false">IFERROR(K7/H7,0)</f>
@@ -11891,7 +11891,7 @@
       </c>
       <c r="AG7" s="43" t="n">
         <f aca="false">IFERROR((K7-AB7-AC7)/H7,0)</f>
-        <v>0.0355992541108663</v>
+        <v>0.0457704695711138</v>
       </c>
       <c r="AH7" s="35"/>
       <c r="AI7" s="34" t="n">
@@ -11997,7 +11997,7 @@
       </c>
       <c r="AB8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$H$37:$H$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N8="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>11880</v>
+        <v>11002.5</v>
       </c>
       <c r="AC8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$C$37:$C$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))</f>
@@ -12005,11 +12005,11 @@
       </c>
       <c r="AD8" s="21" t="n">
         <f aca="false">K8-AB8-W8*12</f>
-        <v>-39154.8085586803</v>
+        <v>-38277.3085586803</v>
       </c>
       <c r="AE8" s="21" t="n">
         <f aca="false">AD8-AC8</f>
-        <v>-42664.8085586803</v>
+        <v>-41787.3085586803</v>
       </c>
       <c r="AF8" s="23" t="n">
         <f aca="false">IFERROR(K8/H8,0)</f>
@@ -12017,7 +12017,7 @@
       </c>
       <c r="AG8" s="23" t="n">
         <f aca="false">IFERROR((K8-AB8-AC8)/H8,0)</f>
-        <v>0.0261509433962264</v>
+        <v>0.0278066037735849</v>
       </c>
       <c r="AH8" s="26"/>
       <c r="AI8" s="13" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="AB6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$H$37:$H$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N6="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>39863.4</v>
+        <v>29965.4</v>
       </c>
       <c r="AC6" s="21" t="n">
         <f aca="false">K6*INDEX(Assumptions!$C$37:$C$38,MATCH(Q6,Assumptions!$B$37:$B$38,0))</f>
@@ -12569,11 +12569,11 @@
       </c>
       <c r="AD6" s="21" t="n">
         <f aca="false">K6-AB6-W6*12</f>
-        <v>-12164.2575558435</v>
+        <v>-2266.25755584351</v>
       </c>
       <c r="AE6" s="21" t="n">
         <f aca="false">AD6-AC6</f>
-        <v>-31960.2575558435</v>
+        <v>-22062.2575558435</v>
       </c>
       <c r="AF6" s="23" t="n">
         <f aca="false">IFERROR(K6/H6,0)</f>
@@ -12581,7 +12581,7 @@
       </c>
       <c r="AG6" s="23" t="n">
         <f aca="false">IFERROR((K6-AB6-AC6)/H6,0)</f>
-        <v>0.0517376315789474</v>
+        <v>0.0647613157894737</v>
       </c>
       <c r="AH6" s="26"/>
       <c r="AI6" s="13"/>
@@ -12687,7 +12687,7 @@
       </c>
       <c r="AB7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$H$37:$H$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N7="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>40200</v>
+        <v>30200</v>
       </c>
       <c r="AC7" s="40" t="n">
         <f aca="false">K7*INDEX(Assumptions!$C$37:$C$38,MATCH(Q7,Assumptions!$B$37:$B$38,0))</f>
@@ -12695,11 +12695,11 @@
       </c>
       <c r="AD7" s="40" t="n">
         <f aca="false">K7-AB7-W7*12</f>
-        <v>-4885.91575316079</v>
+        <v>5114.08424683921</v>
       </c>
       <c r="AE7" s="40" t="n">
         <f aca="false">AD7-AC7</f>
-        <v>-24885.9157531608</v>
+        <v>-14885.9157531608</v>
       </c>
       <c r="AF7" s="43" t="n">
         <f aca="false">IFERROR(K7/H7,0)</f>
@@ -12707,7 +12707,7 @@
       </c>
       <c r="AG7" s="43" t="n">
         <f aca="false">IFERROR((K7-AB7-AC7)/H7,0)</f>
-        <v>0.06368</v>
+        <v>0.07968</v>
       </c>
       <c r="AH7" s="35" t="s">
         <v>369</v>
@@ -12815,7 +12815,7 @@
       </c>
       <c r="AB8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$H$37:$H$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N8="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>26336.04</v>
+        <v>20537.24</v>
       </c>
       <c r="AC8" s="21" t="n">
         <f aca="false">K8*INDEX(Assumptions!$C$37:$C$38,MATCH(Q8,Assumptions!$B$37:$B$38,0))</f>
@@ -12823,11 +12823,11 @@
       </c>
       <c r="AD8" s="21" t="n">
         <f aca="false">K8-AB8-W8*12</f>
-        <v>-36224.2696873884</v>
+        <v>-30425.4696873884</v>
       </c>
       <c r="AE8" s="21" t="n">
         <f aca="false">AD8-AC8</f>
-        <v>-47821.8696873884</v>
+        <v>-42023.0696873884</v>
       </c>
       <c r="AF8" s="23" t="n">
         <f aca="false">IFERROR(K8/H8,0)</f>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="AG8" s="23" t="n">
         <f aca="false">IFERROR((K8-AB8-AC8)/H8,0)</f>
-        <v>0.0299318805970149</v>
+        <v>0.0385868059701493</v>
       </c>
       <c r="AH8" s="26"/>
       <c r="AI8" s="13"/>
@@ -12941,7 +12941,7 @@
       </c>
       <c r="AB9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$H$37:$H$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N9="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>23370</v>
+        <v>18470</v>
       </c>
       <c r="AC9" s="40" t="n">
         <f aca="false">K9*INDEX(Assumptions!$C$37:$C$38,MATCH(Q9,Assumptions!$B$37:$B$38,0))</f>
@@ -12949,11 +12949,11 @@
       </c>
       <c r="AD9" s="40" t="n">
         <f aca="false">K9-AB9-W9*12</f>
-        <v>-40828.3123832872</v>
+        <v>-35928.3123832872</v>
       </c>
       <c r="AE9" s="40" t="n">
         <f aca="false">AD9-AC9</f>
-        <v>-50628.3123832872</v>
+        <v>-45728.3123832872</v>
       </c>
       <c r="AF9" s="43" t="n">
         <f aca="false">IFERROR(K9/H9,0)</f>
@@ -12961,7 +12961,7 @@
       </c>
       <c r="AG9" s="43" t="n">
         <f aca="false">IFERROR((K9-AB9-AC9)/H9,0)</f>
-        <v>0.0243538461538462</v>
+        <v>0.0318923076923077</v>
       </c>
       <c r="AH9" s="35"/>
       <c r="AI9" s="34"/>
@@ -13067,7 +13067,7 @@
       </c>
       <c r="AB10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$H$37:$H$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N10="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>40200</v>
+        <v>30200</v>
       </c>
       <c r="AC10" s="21" t="n">
         <f aca="false">K10*INDEX(Assumptions!$C$37:$C$38,MATCH(Q10,Assumptions!$B$37:$B$38,0))</f>
@@ -13075,11 +13075,11 @@
       </c>
       <c r="AD10" s="21" t="n">
         <f aca="false">K10-AB10-W10*12</f>
-        <v>-16764.6921640458</v>
+        <v>-6764.69216404582</v>
       </c>
       <c r="AE10" s="21" t="n">
         <f aca="false">AD10-AC10</f>
-        <v>-36764.6921640458</v>
+        <v>-26764.6921640458</v>
       </c>
       <c r="AF10" s="23" t="n">
         <f aca="false">IFERROR(K10/H10,0)</f>
@@ -13087,7 +13087,7 @@
       </c>
       <c r="AG10" s="23" t="n">
         <f aca="false">IFERROR((K10-AB10-AC10)/H10,0)</f>
-        <v>0.04975</v>
+        <v>0.06225</v>
       </c>
       <c r="AH10" s="26" t="s">
         <v>383</v>
@@ -13195,7 +13195,7 @@
       </c>
       <c r="AB11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$H$37:$H$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(N11="Y",Assumptions!$C$42,Assumptions!$C$43)</f>
-        <v>19740</v>
+        <v>15940</v>
       </c>
       <c r="AC11" s="40" t="n">
         <f aca="false">K11*INDEX(Assumptions!$C$37:$C$38,MATCH(Q11,Assumptions!$B$37:$B$38,0))</f>
@@ -13203,11 +13203,11 @@
       </c>
       <c r="AD11" s="40" t="n">
         <f aca="false">K11-AB11-W11*12</f>
-        <v>-40045.2878847056</v>
+        <v>-36245.2878847056</v>
       </c>
       <c r="AE11" s="40" t="n">
         <f aca="false">AD11-AC11</f>
-        <v>-47645.2878847056</v>
+        <v>-43845.2878847056</v>
       </c>
       <c r="AF11" s="43" t="n">
         <f aca="false">IFERROR(K11/H11,0)</f>
@@ -13215,7 +13215,7 @@
       </c>
       <c r="AG11" s="43" t="n">
         <f aca="false">IFERROR((K11-AB11-AC11)/H11,0)</f>
-        <v>0.0199252336448598</v>
+        <v>0.0270280373831776</v>
       </c>
       <c r="AH11" s="35"/>
       <c r="AI11" s="34" t="n">
@@ -13588,15 +13588,15 @@
       </c>
       <c r="M5" s="21" t="n">
         <f aca="false">E5-(E5*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I5*12</f>
-        <v>-7039.77197979741</v>
+        <v>1460.22802020259</v>
       </c>
       <c r="N5" s="21" t="n">
         <f aca="false">M5-E5*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-24039.7719797974</v>
+        <v>-15539.7719797974</v>
       </c>
       <c r="O5" s="23" t="n">
         <f aca="false">IFERROR(M5/L5,0)</f>
-        <v>-0.0598620066309303</v>
+        <v>0.0124169049336955</v>
       </c>
       <c r="P5" s="47" t="s">
         <v>420</v>
@@ -13652,15 +13652,15 @@
       </c>
       <c r="M6" s="21" t="n">
         <f aca="false">E6-(E6*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I6*12</f>
-        <v>-3831.68451483207</v>
+        <v>4668.31548516793</v>
       </c>
       <c r="N6" s="21" t="n">
         <f aca="false">M6-E6*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-20831.6845148321</v>
+        <v>-12331.6845148321</v>
       </c>
       <c r="O6" s="23" t="n">
         <f aca="false">IFERROR(M6/L6,0)</f>
-        <v>-0.0263165145249455</v>
+        <v>0.0320626063541753</v>
       </c>
       <c r="P6" s="23" t="n">
         <f aca="false">IFERROR((M6-M5)/(L6-L5),0)</f>
@@ -13717,15 +13717,15 @@
       </c>
       <c r="M7" s="21" t="n">
         <f aca="false">E7-(E7*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I7*12</f>
-        <v>-1141.71933608533</v>
+        <v>7358.28066391467</v>
       </c>
       <c r="N7" s="21" t="n">
         <f aca="false">M7-E7*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-18141.7193360853</v>
+        <v>-9641.71933608533</v>
       </c>
       <c r="O7" s="23" t="n">
         <f aca="false">IFERROR(M7/L7,0)</f>
-        <v>-0.00657672428620584</v>
+        <v>0.0423864093543472</v>
       </c>
       <c r="P7" s="23" t="n">
         <f aca="false">IFERROR((M7-M6)/(L7-L6),0)</f>
@@ -13782,15 +13782,15 @@
       </c>
       <c r="M9" s="21" t="n">
         <f aca="false">E9-(E9*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$7="Y",Assumptions!$C$42,Assumptions!$C$43))-I9*12</f>
-        <v>-5067.31269769074</v>
+        <v>2232.68730230926</v>
       </c>
       <c r="N9" s="21" t="n">
         <f aca="false">M9-E9*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$7,Assumptions!$B$37:$B$38,0))</f>
-        <v>-19667.3126976907</v>
+        <v>-12367.3126976907</v>
       </c>
       <c r="O9" s="23" t="n">
         <f aca="false">IFERROR(M9/L9,0)</f>
-        <v>-0.0458995715370538</v>
+        <v>0.0202236168687433</v>
       </c>
       <c r="P9" s="47" t="s">
         <v>420</v>
@@ -13846,15 +13846,15 @@
       </c>
       <c r="M10" s="21" t="n">
         <f aca="false">E10-(E10*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$7="Y",Assumptions!$C$42,Assumptions!$C$43))-I10*12</f>
-        <v>-2432.09799432634</v>
+        <v>4867.90200567366</v>
       </c>
       <c r="N10" s="21" t="n">
         <f aca="false">M10-E10*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$7,Assumptions!$B$37:$B$38,0))</f>
-        <v>-17032.0979943263</v>
+        <v>-9732.09799432635</v>
       </c>
       <c r="O10" s="23" t="n">
         <f aca="false">IFERROR(M10/L10,0)</f>
-        <v>-0.0182316191478737</v>
+        <v>0.036491019532786</v>
       </c>
       <c r="P10" s="23" t="n">
         <f aca="false">IFERROR((M10-M9)/(L10-L9),0)</f>
@@ -13911,15 +13911,15 @@
       </c>
       <c r="M11" s="21" t="n">
         <f aca="false">E11-(E11*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$7="Y",Assumptions!$C$42,Assumptions!$C$43))-I11*12</f>
-        <v>-222.483740355812</v>
+        <v>7077.51625964419</v>
       </c>
       <c r="N11" s="21" t="n">
         <f aca="false">M11-E11*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$7,Assumptions!$B$37:$B$38,0))</f>
-        <v>-14822.4837403558</v>
+        <v>-7522.48374035581</v>
       </c>
       <c r="O11" s="23" t="n">
         <f aca="false">IFERROR(M11/L11,0)</f>
-        <v>-0.00142253030918038</v>
+        <v>0.0452526615066764</v>
       </c>
       <c r="P11" s="23" t="n">
         <f aca="false">IFERROR((M11-M10)/(L11-L10),0)</f>
@@ -13976,15 +13976,15 @@
       </c>
       <c r="M13" s="21" t="n">
         <f aca="false">E13-(E13*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$8="Y",Assumptions!$C$42,Assumptions!$C$43))-I13*12</f>
-        <v>-7644.75569264008</v>
+        <v>1255.24430735992</v>
       </c>
       <c r="N13" s="21" t="n">
         <f aca="false">M13-E13*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$8,Assumptions!$B$37:$B$38,0))</f>
-        <v>-25444.7556926401</v>
+        <v>-16544.7556926401</v>
       </c>
       <c r="O13" s="23" t="n">
         <f aca="false">IFERROR(M13/L13,0)</f>
-        <v>-0.0606726642273022</v>
+        <v>0.00996225640761842</v>
       </c>
       <c r="P13" s="47" t="s">
         <v>420</v>
@@ -14040,15 +14040,15 @@
       </c>
       <c r="M14" s="21" t="n">
         <f aca="false">E14-(E14*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$8="Y",Assumptions!$C$42,Assumptions!$C$43))-I14*12</f>
-        <v>-4207.51912303436</v>
+        <v>4692.48087696564</v>
       </c>
       <c r="N14" s="21" t="n">
         <f aca="false">M14-E14*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$8,Assumptions!$B$37:$B$38,0))</f>
-        <v>-22007.5191230344</v>
+        <v>-13107.5191230344</v>
       </c>
       <c r="O14" s="23" t="n">
         <f aca="false">IFERROR(M14/L14,0)</f>
-        <v>-0.0269712764297075</v>
+        <v>0.0300800056215746</v>
       </c>
       <c r="P14" s="23" t="n">
         <f aca="false">IFERROR((M14-M13)/(L14-L13),0)</f>
@@ -14105,15 +14105,15 @@
       </c>
       <c r="M15" s="21" t="n">
         <f aca="false">E15-(E15*INDEX(Assumptions!$H$37:$H$38,MATCH('Manatee-Sarasota'!$Q$8,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Manatee-Sarasota'!$N$8="Y",Assumptions!$C$42,Assumptions!$C$43))-I15*12</f>
-        <v>-1325.41357437715</v>
+        <v>7574.58642562285</v>
       </c>
       <c r="N15" s="21" t="n">
         <f aca="false">M15-E15*INDEX(Assumptions!$C$37:$C$38,MATCH('Manatee-Sarasota'!$Q$8,Assumptions!$B$37:$B$38,0))</f>
-        <v>-19125.4135743771</v>
+        <v>-10225.4135743771</v>
       </c>
       <c r="O15" s="23" t="n">
         <f aca="false">IFERROR(M15/L15,0)</f>
-        <v>-0.0071258794321352</v>
+        <v>0.0407235829334562</v>
       </c>
       <c r="P15" s="23" t="n">
         <f aca="false">IFERROR((M15-M14)/(L15-L14),0)</f>
@@ -14170,15 +14170,15 @@
       </c>
       <c r="M17" s="21" t="n">
         <f aca="false">E17-(E17*INDEX(Assumptions!$H$37:$H$38,MATCH(Pinellas!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(Pinellas!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I17*12</f>
-        <v>-10745.4275182174</v>
+        <v>-3645.4275182174</v>
       </c>
       <c r="N17" s="21" t="n">
         <f aca="false">M17-E17*INDEX(Assumptions!$C$37:$C$38,MATCH(Pinellas!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-24945.4275182174</v>
+        <v>-17845.4275182174</v>
       </c>
       <c r="O17" s="23" t="n">
         <f aca="false">IFERROR(M17/L17,0)</f>
-        <v>-0.0923146694004932</v>
+        <v>-0.03131810582661</v>
       </c>
       <c r="P17" s="47" t="s">
         <v>420</v>
@@ -14234,15 +14234,15 @@
       </c>
       <c r="M18" s="21" t="n">
         <f aca="false">E18-(E18*INDEX(Assumptions!$H$37:$H$38,MATCH(Pinellas!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(Pinellas!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I18*12</f>
-        <v>-7966.99462445278</v>
+        <v>-866.994624452775</v>
       </c>
       <c r="N18" s="21" t="n">
         <f aca="false">M18-E18*INDEX(Assumptions!$C$37:$C$38,MATCH(Pinellas!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-22166.9946244528</v>
+        <v>-15066.9946244528</v>
       </c>
       <c r="O18" s="23" t="n">
         <f aca="false">IFERROR(M18/L18,0)</f>
-        <v>-0.0566441139314097</v>
+        <v>-0.00616419924957536</v>
       </c>
       <c r="P18" s="23" t="n">
         <f aca="false">IFERROR((M18-M17)/(L18-L17),0)</f>
@@ -14299,15 +14299,15 @@
       </c>
       <c r="M19" s="21" t="n">
         <f aca="false">E19-(E19*INDEX(Assumptions!$H$37:$H$38,MATCH(Pinellas!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(Pinellas!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I19*12</f>
-        <v>-5637.29263928819</v>
+        <v>1462.70736071181</v>
       </c>
       <c r="N19" s="21" t="n">
         <f aca="false">M19-E19*INDEX(Assumptions!$C$37:$C$38,MATCH(Pinellas!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-19837.2926392882</v>
+        <v>-12737.2926392882</v>
       </c>
       <c r="O19" s="23" t="n">
         <f aca="false">IFERROR(M19/L19,0)</f>
-        <v>-0.03418612880102</v>
+        <v>0.00887026901583874</v>
       </c>
       <c r="P19" s="23" t="n">
         <f aca="false">IFERROR((M19-M18)/(L19-L18),0)</f>
@@ -14364,15 +14364,15 @@
       </c>
       <c r="M21" s="21" t="n">
         <f aca="false">E21-(E21*INDEX(Assumptions!$H$37:$H$38,MATCH(Pinellas!$Q$7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(Pinellas!$N$7="Y",Assumptions!$C$42,Assumptions!$C$43))-I21*12</f>
-        <v>-1365.4275182174</v>
+        <v>7134.5724817826</v>
       </c>
       <c r="N21" s="21" t="n">
         <f aca="false">M21-E21*INDEX(Assumptions!$C$37:$C$38,MATCH(Pinellas!$Q$7,Assumptions!$B$37:$B$38,0))</f>
-        <v>-18365.4275182174</v>
+        <v>-9865.4275182174</v>
       </c>
       <c r="O21" s="23" t="n">
         <f aca="false">IFERROR(M21/L21,0)</f>
-        <v>-0.0117304769606306</v>
+        <v>0.0612935780221873</v>
       </c>
       <c r="P21" s="47" t="s">
         <v>420</v>
@@ -14428,15 +14428,15 @@
       </c>
       <c r="M22" s="21" t="n">
         <f aca="false">E22-(E22*INDEX(Assumptions!$H$37:$H$38,MATCH(Pinellas!$Q$7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(Pinellas!$N$7="Y",Assumptions!$C$42,Assumptions!$C$43))-I22*12</f>
-        <v>1413.00537554723</v>
+        <v>9913.00537554723</v>
       </c>
       <c r="N22" s="21" t="n">
         <f aca="false">M22-E22*INDEX(Assumptions!$C$37:$C$38,MATCH(Pinellas!$Q$7,Assumptions!$B$37:$B$38,0))</f>
-        <v>-15586.9946244528</v>
+        <v>-7086.99462445278</v>
       </c>
       <c r="O22" s="23" t="n">
         <f aca="false">IFERROR(M22/L22,0)</f>
-        <v>0.0100462522257179</v>
+        <v>0.0704799529011534</v>
       </c>
       <c r="P22" s="23" t="n">
         <f aca="false">IFERROR((M22-M21)/(L22-L21),0)</f>
@@ -14493,15 +14493,15 @@
       </c>
       <c r="M23" s="21" t="n">
         <f aca="false">E23-(E23*INDEX(Assumptions!$H$37:$H$38,MATCH(Pinellas!$Q$7,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF(Pinellas!$N$7="Y",Assumptions!$C$42,Assumptions!$C$43))-I23*12</f>
-        <v>3742.70736071181</v>
+        <v>12242.7073607118</v>
       </c>
       <c r="N23" s="21" t="n">
         <f aca="false">M23-E23*INDEX(Assumptions!$C$37:$C$38,MATCH(Pinellas!$Q$7,Assumptions!$B$37:$B$38,0))</f>
-        <v>-13257.2926392882</v>
+        <v>-4757.29263928819</v>
       </c>
       <c r="O23" s="23" t="n">
         <f aca="false">IFERROR(M23/L23,0)</f>
-        <v>0.0226968305682948</v>
+        <v>0.0742432223208721</v>
       </c>
       <c r="P23" s="23" t="n">
         <f aca="false">IFERROR((M23-M22)/(L23-L22),0)</f>
@@ -14558,15 +14558,15 @@
       </c>
       <c r="M25" s="21" t="n">
         <f aca="false">E25-(E25*INDEX(Assumptions!$H$37:$H$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Monroe (Keys)'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I25*12</f>
-        <v>-16518.0905440108</v>
+        <v>-6620.09054401076</v>
       </c>
       <c r="N25" s="21" t="n">
         <f aca="false">M25-E25*INDEX(Assumptions!$C$37:$C$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-36314.0905440108</v>
+        <v>-26416.0905440108</v>
       </c>
       <c r="O25" s="23" t="n">
         <f aca="false">IFERROR(M25/L25,0)</f>
-        <v>-0.0905597069298836</v>
+        <v>-0.0362943560526906</v>
       </c>
       <c r="P25" s="47" t="s">
         <v>420</v>
@@ -14622,15 +14622,15 @@
       </c>
       <c r="M26" s="21" t="n">
         <f aca="false">E26-(E26*INDEX(Assumptions!$H$37:$H$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Monroe (Keys)'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I26*12</f>
-        <v>-12164.2575558435</v>
+        <v>-2266.25755584351</v>
       </c>
       <c r="N26" s="21" t="n">
         <f aca="false">M26-E26*INDEX(Assumptions!$C$37:$C$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-31960.2575558435</v>
+        <v>-22062.2575558435</v>
       </c>
       <c r="O26" s="23" t="n">
         <f aca="false">IFERROR(M26/L26,0)</f>
-        <v>-0.0551917311971121</v>
+        <v>-0.0102824752987455</v>
       </c>
       <c r="P26" s="23" t="n">
         <f aca="false">IFERROR((M26-M25)/(L26-L25),0)</f>
@@ -14687,15 +14687,15 @@
       </c>
       <c r="M27" s="21" t="n">
         <f aca="false">E27-(E27*INDEX(Assumptions!$H$37:$H$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))+Assumptions!$C$41+IF('Monroe (Keys)'!$N$6="Y",Assumptions!$C$42,Assumptions!$C$43))-I27*12</f>
-        <v>-8513.59052754439</v>
+        <v>1384.40947245562</v>
       </c>
       <c r="N27" s="21" t="n">
         <f aca="false">M27-E27*INDEX(Assumptions!$C$37:$C$38,MATCH('Monroe (Keys)'!$Q$6,Assumptions!$B$37:$B$38,0))</f>
-        <v>-28309.5905275444</v>
+        <v>-18411.5905275444</v>
       </c>
       <c r="O27" s="23" t="n">
         <f aca="false">IFERROR(M27/L27,0)</f>
-        <v>-0.0329473317629427</v>
+        <v>0.00535762179742887</v>
       </c>
       <c r="P27" s="23" t="n">
         <f aca="false">IFERROR((M27-M26)/(L27-L26),0)</f>

</xml_diff>